<commit_message>
Update Swordsman (검사) full gear recipes and set mining locations for 현빙 and 지옥석
</commit_message>
<xml_diff>
--- a/dream01.xlsx
+++ b/dream01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\Dream\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A224365-7B68-424B-BF0D-E332B9D0E864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD338E2A-8BB7-448B-BEC2-E83A5FAE55C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2410" yWindow="430" windowWidth="19710" windowHeight="19840" tabRatio="703" xr2:uid="{DC656F52-3D86-40C7-8433-EB14A2C834F9}"/>
+    <workbookView xWindow="2410" yWindow="430" windowWidth="19710" windowHeight="19840" tabRatio="703" activeTab="5" xr2:uid="{DC656F52-3D86-40C7-8433-EB14A2C834F9}"/>
   </bookViews>
   <sheets>
     <sheet name="보스" sheetId="3" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2866" uniqueCount="624">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2943" uniqueCount="629">
   <si>
     <t>Lv.1</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -2492,14 +2492,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>봉황 화염</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>내면의 심연석</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>진홍의 살육</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -2537,6 +2529,34 @@
   </si>
   <si>
     <t>네크로맨서 장화</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>심연의 마나석</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>지옥불-성스러운 악마의 화염 반지</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>아즈모단-마왕의 반지</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>지옥 지배자의 반지</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>암흑 반지</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>용암 화산-채광</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>운설산-채광</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -4264,7 +4284,7 @@
         <v>503</v>
       </c>
       <c r="E55" s="27" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.45">
@@ -4297,30 +4317,30 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A58" s="27" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="B58" s="27">
         <v>300</v>
       </c>
       <c r="C58" s="27" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="D58" s="27" t="s">
         <v>157</v>
       </c>
       <c r="E58" s="27" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A59" s="27" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="B59" s="27">
         <v>300</v>
       </c>
       <c r="C59" s="27" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="D59" s="27" t="s">
         <v>157</v>
@@ -17179,7 +17199,9 @@
       <c r="D165" s="8">
         <v>25</v>
       </c>
-      <c r="E165" s="8"/>
+      <c r="E165" s="8" t="s">
+        <v>627</v>
+      </c>
       <c r="F165" s="8"/>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.45">
@@ -18013,7 +18035,7 @@
         <v>12</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>517</v>
+        <v>628</v>
       </c>
       <c r="F30" s="8"/>
     </row>
@@ -20254,7 +20276,7 @@
         <v>611</v>
       </c>
       <c r="C5" s="25" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="D5" s="25">
         <v>1</v>
@@ -20268,7 +20290,7 @@
       <c r="A6" s="42"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="D6" s="8">
         <v>1</v>
@@ -20292,7 +20314,7 @@
       <c r="A8" s="42"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="D8" s="8">
         <v>1</v>
@@ -20339,10 +20361,10 @@
     <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" s="42"/>
       <c r="B12" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="D12" s="8">
         <v>1</v>
@@ -20427,10 +20449,10 @@
     <row r="19" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A19" s="42"/>
       <c r="B19" s="8" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="D19" s="8">
         <v>1</v>
@@ -20444,7 +20466,7 @@
       <c r="A20" s="42"/>
       <c r="B20" s="8"/>
       <c r="C20" s="8" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="D20" s="8">
         <v>1</v>
@@ -21023,17 +21045,23 @@
         <v>481</v>
       </c>
       <c r="B70" s="8" t="s">
-        <v>612</v>
-      </c>
-      <c r="C70" s="8"/>
+        <v>482</v>
+      </c>
+      <c r="C70" s="8" t="s">
+        <v>483</v>
+      </c>
       <c r="D70" s="8"/>
       <c r="E70" s="8"/>
-      <c r="F70" s="8"/>
+      <c r="F70" s="8">
+        <v>380</v>
+      </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A71" s="41"/>
       <c r="B71" s="8"/>
-      <c r="C71" s="8"/>
+      <c r="C71" s="8" t="s">
+        <v>484</v>
+      </c>
       <c r="D71" s="8"/>
       <c r="E71" s="8"/>
       <c r="F71" s="8"/>
@@ -21041,159 +21069,243 @@
     <row r="72" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A72" s="41"/>
       <c r="B72" s="8"/>
-      <c r="C72" s="8"/>
-      <c r="D72" s="8"/>
+      <c r="C72" s="8" t="s">
+        <v>485</v>
+      </c>
+      <c r="D72" s="8">
+        <v>1</v>
+      </c>
       <c r="E72" s="8"/>
       <c r="F72" s="8"/>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A73" s="41"/>
       <c r="B73" s="8"/>
-      <c r="C73" s="8"/>
-      <c r="D73" s="8"/>
+      <c r="C73" s="8" t="s">
+        <v>486</v>
+      </c>
+      <c r="D73" s="8">
+        <v>1</v>
+      </c>
       <c r="E73" s="8"/>
       <c r="F73" s="8"/>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A74" s="41"/>
       <c r="B74" s="8"/>
-      <c r="C74" s="8"/>
-      <c r="D74" s="8"/>
+      <c r="C74" s="8" t="s">
+        <v>460</v>
+      </c>
+      <c r="D74" s="8">
+        <v>1</v>
+      </c>
       <c r="E74" s="8"/>
       <c r="F74" s="8"/>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A75" s="41"/>
       <c r="B75" s="8"/>
-      <c r="C75" s="8"/>
-      <c r="D75" s="8"/>
+      <c r="C75" s="8" t="s">
+        <v>487</v>
+      </c>
+      <c r="D75" s="8">
+        <v>1</v>
+      </c>
       <c r="E75" s="8"/>
       <c r="F75" s="8"/>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A76" s="41"/>
       <c r="B76" s="8"/>
-      <c r="C76" s="8"/>
-      <c r="D76" s="8"/>
+      <c r="C76" s="8" t="s">
+        <v>419</v>
+      </c>
+      <c r="D76" s="8">
+        <v>1</v>
+      </c>
       <c r="E76" s="8"/>
       <c r="F76" s="8"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A77" s="41"/>
-      <c r="B77" s="8"/>
-      <c r="C77" s="8"/>
+      <c r="B77" s="8" t="s">
+        <v>483</v>
+      </c>
+      <c r="C77" s="8" t="s">
+        <v>492</v>
+      </c>
       <c r="D77" s="8"/>
       <c r="E77" s="8"/>
-      <c r="F77" s="8"/>
+      <c r="F77" s="8">
+        <v>360</v>
+      </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A78" s="41"/>
       <c r="B78" s="8"/>
-      <c r="C78" s="8"/>
-      <c r="D78" s="8"/>
+      <c r="C78" s="8" t="s">
+        <v>493</v>
+      </c>
+      <c r="D78" s="8">
+        <v>1</v>
+      </c>
       <c r="E78" s="8"/>
       <c r="F78" s="8"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A79" s="41"/>
       <c r="B79" s="8"/>
-      <c r="C79" s="8"/>
-      <c r="D79" s="8"/>
+      <c r="C79" s="8" t="s">
+        <v>420</v>
+      </c>
+      <c r="D79" s="8">
+        <v>1</v>
+      </c>
       <c r="E79" s="8"/>
       <c r="F79" s="8"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A80" s="41"/>
       <c r="B80" s="8"/>
-      <c r="C80" s="8"/>
-      <c r="D80" s="8"/>
+      <c r="C80" s="8" t="s">
+        <v>463</v>
+      </c>
+      <c r="D80" s="8">
+        <v>1</v>
+      </c>
       <c r="E80" s="8"/>
       <c r="F80" s="8"/>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A81" s="41"/>
       <c r="B81" s="8"/>
-      <c r="C81" s="8"/>
-      <c r="D81" s="8"/>
+      <c r="C81" s="8" t="s">
+        <v>494</v>
+      </c>
+      <c r="D81" s="8">
+        <v>1</v>
+      </c>
       <c r="E81" s="8"/>
       <c r="F81" s="8"/>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A82" s="41"/>
       <c r="B82" s="8"/>
-      <c r="C82" s="8"/>
-      <c r="D82" s="8"/>
+      <c r="C82" s="8" t="s">
+        <v>368</v>
+      </c>
+      <c r="D82" s="8">
+        <v>1</v>
+      </c>
       <c r="E82" s="8"/>
       <c r="F82" s="8"/>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A83" s="41"/>
       <c r="B83" s="8"/>
-      <c r="C83" s="8"/>
-      <c r="D83" s="8"/>
+      <c r="C83" s="8" t="s">
+        <v>495</v>
+      </c>
+      <c r="D83" s="8">
+        <v>1</v>
+      </c>
       <c r="E83" s="8"/>
       <c r="F83" s="8"/>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A84" s="41"/>
-      <c r="B84" s="8"/>
-      <c r="C84" s="8"/>
+      <c r="B84" s="8" t="s">
+        <v>492</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>496</v>
+      </c>
       <c r="D84" s="8"/>
       <c r="E84" s="8"/>
-      <c r="F84" s="8"/>
+      <c r="F84" s="8">
+        <v>340</v>
+      </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A85" s="41"/>
       <c r="B85" s="8"/>
-      <c r="C85" s="8"/>
-      <c r="D85" s="8"/>
+      <c r="C85" s="8" t="s">
+        <v>497</v>
+      </c>
+      <c r="D85" s="8">
+        <v>1</v>
+      </c>
       <c r="E85" s="8"/>
       <c r="F85" s="8"/>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A86" s="41"/>
       <c r="B86" s="8"/>
-      <c r="C86" s="8"/>
-      <c r="D86" s="8"/>
+      <c r="C86" s="8" t="s">
+        <v>494</v>
+      </c>
+      <c r="D86" s="8">
+        <v>1</v>
+      </c>
       <c r="E86" s="8"/>
       <c r="F86" s="8"/>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A87" s="41"/>
       <c r="B87" s="8"/>
-      <c r="C87" s="8"/>
-      <c r="D87" s="8"/>
+      <c r="C87" s="8" t="s">
+        <v>498</v>
+      </c>
+      <c r="D87" s="8">
+        <v>1</v>
+      </c>
       <c r="E87" s="8"/>
       <c r="F87" s="8"/>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A88" s="41"/>
       <c r="B88" s="8"/>
-      <c r="C88" s="8"/>
-      <c r="D88" s="8"/>
+      <c r="C88" s="8" t="s">
+        <v>436</v>
+      </c>
+      <c r="D88" s="8">
+        <v>1</v>
+      </c>
       <c r="E88" s="8"/>
       <c r="F88" s="8"/>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A89" s="41"/>
       <c r="B89" s="8"/>
-      <c r="C89" s="8"/>
-      <c r="D89" s="8"/>
+      <c r="C89" s="8" t="s">
+        <v>499</v>
+      </c>
+      <c r="D89" s="8">
+        <v>1</v>
+      </c>
       <c r="E89" s="8"/>
       <c r="F89" s="8"/>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A90" s="41"/>
-      <c r="B90" s="8"/>
-      <c r="C90" s="8"/>
+      <c r="B90" s="8" t="s">
+        <v>496</v>
+      </c>
+      <c r="C90" s="8" t="s">
+        <v>500</v>
+      </c>
       <c r="D90" s="8"/>
       <c r="E90" s="8"/>
-      <c r="F90" s="8"/>
+      <c r="F90" s="8">
+        <v>320</v>
+      </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A91" s="41"/>
       <c r="B91" s="8"/>
-      <c r="C91" s="8"/>
+      <c r="C91" s="8" t="s">
+        <v>401</v>
+      </c>
       <c r="D91" s="8"/>
       <c r="E91" s="8"/>
       <c r="F91" s="8"/>
@@ -21201,7 +21313,9 @@
     <row r="92" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A92" s="41"/>
       <c r="B92" s="8"/>
-      <c r="C92" s="8"/>
+      <c r="C92" s="8" t="s">
+        <v>368</v>
+      </c>
       <c r="D92" s="8"/>
       <c r="E92" s="8"/>
       <c r="F92" s="8"/>
@@ -21209,152 +21323,232 @@
     <row r="93" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A93" s="41"/>
       <c r="B93" s="8"/>
-      <c r="C93" s="8"/>
+      <c r="C93" s="8" t="s">
+        <v>370</v>
+      </c>
       <c r="D93" s="8"/>
       <c r="E93" s="8"/>
       <c r="F93" s="8"/>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A94" s="41"/>
-      <c r="B94" s="8"/>
-      <c r="C94" s="8"/>
+      <c r="B94" s="8" t="s">
+        <v>484</v>
+      </c>
+      <c r="C94" s="8" t="s">
+        <v>504</v>
+      </c>
       <c r="D94" s="8"/>
       <c r="E94" s="8"/>
-      <c r="F94" s="8"/>
+      <c r="F94" s="8">
+        <v>360</v>
+      </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A95" s="41"/>
       <c r="B95" s="8"/>
-      <c r="C95" s="8"/>
-      <c r="D95" s="8"/>
+      <c r="C95" s="8" t="s">
+        <v>437</v>
+      </c>
+      <c r="D95" s="8">
+        <v>1</v>
+      </c>
       <c r="E95" s="8"/>
       <c r="F95" s="8"/>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A96" s="41"/>
       <c r="B96" s="8"/>
-      <c r="C96" s="8"/>
-      <c r="D96" s="8"/>
+      <c r="C96" s="8" t="s">
+        <v>505</v>
+      </c>
+      <c r="D96" s="8">
+        <v>1</v>
+      </c>
       <c r="E96" s="8"/>
       <c r="F96" s="8"/>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A97" s="41"/>
       <c r="B97" s="8"/>
-      <c r="C97" s="8"/>
-      <c r="D97" s="8"/>
+      <c r="C97" s="8" t="s">
+        <v>463</v>
+      </c>
+      <c r="D97" s="8">
+        <v>1</v>
+      </c>
       <c r="E97" s="8"/>
       <c r="F97" s="8"/>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A98" s="41"/>
       <c r="B98" s="8"/>
-      <c r="C98" s="8"/>
-      <c r="D98" s="8"/>
+      <c r="C98" s="8" t="s">
+        <v>506</v>
+      </c>
+      <c r="D98" s="8">
+        <v>1</v>
+      </c>
       <c r="E98" s="8"/>
       <c r="F98" s="8"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A99" s="41"/>
       <c r="B99" s="8"/>
-      <c r="C99" s="8"/>
-      <c r="D99" s="8"/>
+      <c r="C99" s="8" t="s">
+        <v>368</v>
+      </c>
+      <c r="D99" s="8">
+        <v>1</v>
+      </c>
       <c r="E99" s="8"/>
       <c r="F99" s="8"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A100" s="41"/>
       <c r="B100" s="8"/>
-      <c r="C100" s="8"/>
-      <c r="D100" s="8"/>
+      <c r="C100" s="8" t="s">
+        <v>334</v>
+      </c>
+      <c r="D100" s="8">
+        <v>1</v>
+      </c>
       <c r="E100" s="8"/>
       <c r="F100" s="8"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A101" s="41"/>
-      <c r="B101" s="8"/>
-      <c r="C101" s="8"/>
+      <c r="B101" s="8" t="s">
+        <v>504</v>
+      </c>
+      <c r="C101" s="8" t="s">
+        <v>507</v>
+      </c>
       <c r="D101" s="8"/>
       <c r="E101" s="8"/>
-      <c r="F101" s="8"/>
+      <c r="F101" s="8">
+        <v>340</v>
+      </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A102" s="41"/>
       <c r="B102" s="8"/>
-      <c r="C102" s="8"/>
-      <c r="D102" s="8"/>
+      <c r="C102" s="8" t="s">
+        <v>508</v>
+      </c>
+      <c r="D102" s="8">
+        <v>1</v>
+      </c>
       <c r="E102" s="8"/>
       <c r="F102" s="8"/>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A103" s="41"/>
       <c r="B103" s="8"/>
-      <c r="C103" s="8"/>
-      <c r="D103" s="8"/>
+      <c r="C103" s="8" t="s">
+        <v>497</v>
+      </c>
+      <c r="D103" s="8">
+        <v>1</v>
+      </c>
       <c r="E103" s="8"/>
       <c r="F103" s="8"/>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A104" s="41"/>
       <c r="B104" s="8"/>
-      <c r="C104" s="8"/>
-      <c r="D104" s="8"/>
+      <c r="C104" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="D104" s="8">
+        <v>1</v>
+      </c>
       <c r="E104" s="8"/>
       <c r="F104" s="8"/>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A105" s="41"/>
       <c r="B105" s="8"/>
-      <c r="C105" s="8"/>
-      <c r="D105" s="8"/>
+      <c r="C105" s="8" t="s">
+        <v>401</v>
+      </c>
+      <c r="D105" s="8">
+        <v>1</v>
+      </c>
       <c r="E105" s="8"/>
       <c r="F105" s="8"/>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A106" s="41"/>
       <c r="B106" s="8"/>
-      <c r="C106" s="8"/>
-      <c r="D106" s="8"/>
+      <c r="C106" s="8" t="s">
+        <v>471</v>
+      </c>
+      <c r="D106" s="8">
+        <v>1</v>
+      </c>
       <c r="E106" s="8"/>
       <c r="F106" s="8"/>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A107" s="41"/>
-      <c r="B107" s="8"/>
-      <c r="C107" s="8"/>
-      <c r="D107" s="8"/>
+      <c r="B107" s="8" t="s">
+        <v>507</v>
+      </c>
+      <c r="C107" s="8" t="s">
+        <v>509</v>
+      </c>
+      <c r="D107" s="8">
+        <v>1</v>
+      </c>
       <c r="E107" s="8"/>
       <c r="F107" s="8"/>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A108" s="41"/>
       <c r="B108" s="8"/>
-      <c r="C108" s="8"/>
-      <c r="D108" s="8"/>
+      <c r="C108" s="8" t="s">
+        <v>510</v>
+      </c>
+      <c r="D108" s="8">
+        <v>1</v>
+      </c>
       <c r="E108" s="8"/>
       <c r="F108" s="8"/>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A109" s="41"/>
       <c r="B109" s="8"/>
-      <c r="C109" s="8"/>
-      <c r="D109" s="8"/>
+      <c r="C109" s="8" t="s">
+        <v>500</v>
+      </c>
+      <c r="D109" s="8">
+        <v>1</v>
+      </c>
       <c r="E109" s="8"/>
       <c r="F109" s="8"/>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A110" s="41"/>
       <c r="B110" s="8"/>
-      <c r="C110" s="8"/>
-      <c r="D110" s="8"/>
+      <c r="C110" s="8" t="s">
+        <v>401</v>
+      </c>
+      <c r="D110" s="8">
+        <v>1</v>
+      </c>
       <c r="E110" s="8"/>
       <c r="F110" s="8"/>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A111" s="41"/>
       <c r="B111" s="8"/>
-      <c r="C111" s="8"/>
-      <c r="D111" s="8"/>
+      <c r="C111" s="8" t="s">
+        <v>471</v>
+      </c>
+      <c r="D111" s="8">
+        <v>1</v>
+      </c>
       <c r="E111" s="8"/>
       <c r="F111" s="8"/>
     </row>
@@ -22453,202 +22647,316 @@
         <v>544</v>
       </c>
       <c r="B195" s="8" t="s">
-        <v>613</v>
-      </c>
-      <c r="C195" s="8"/>
-      <c r="D195" s="8"/>
+        <v>622</v>
+      </c>
+      <c r="C195" s="8" t="s">
+        <v>572</v>
+      </c>
+      <c r="D195" s="8">
+        <v>1</v>
+      </c>
       <c r="E195" s="8"/>
-      <c r="F195" s="8"/>
+      <c r="F195" s="8">
+        <v>380</v>
+      </c>
     </row>
     <row r="196" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A196" s="41"/>
       <c r="B196" s="8"/>
-      <c r="C196" s="8"/>
-      <c r="D196" s="8"/>
+      <c r="C196" s="8" t="s">
+        <v>623</v>
+      </c>
+      <c r="D196" s="8">
+        <v>1</v>
+      </c>
       <c r="E196" s="8"/>
       <c r="F196" s="8"/>
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A197" s="41"/>
       <c r="B197" s="8"/>
-      <c r="C197" s="8"/>
-      <c r="D197" s="8"/>
+      <c r="C197" s="8" t="s">
+        <v>491</v>
+      </c>
+      <c r="D197" s="8">
+        <v>1</v>
+      </c>
       <c r="E197" s="8"/>
       <c r="F197" s="8"/>
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A198" s="41"/>
       <c r="B198" s="8"/>
-      <c r="C198" s="8"/>
-      <c r="D198" s="8"/>
+      <c r="C198" s="8" t="s">
+        <v>442</v>
+      </c>
+      <c r="D198" s="8">
+        <v>1</v>
+      </c>
       <c r="E198" s="8"/>
       <c r="F198" s="8"/>
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A199" s="41"/>
       <c r="B199" s="8"/>
-      <c r="C199" s="8"/>
-      <c r="D199" s="8"/>
+      <c r="C199" s="8" t="s">
+        <v>461</v>
+      </c>
+      <c r="D199" s="8">
+        <v>1</v>
+      </c>
       <c r="E199" s="8"/>
       <c r="F199" s="8"/>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A200" s="41"/>
       <c r="B200" s="8"/>
-      <c r="C200" s="8"/>
-      <c r="D200" s="8"/>
+      <c r="C200" s="8" t="s">
+        <v>463</v>
+      </c>
+      <c r="D200" s="8">
+        <v>1</v>
+      </c>
       <c r="E200" s="8"/>
       <c r="F200" s="8"/>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A201" s="41"/>
       <c r="B201" s="8"/>
-      <c r="C201" s="8"/>
-      <c r="D201" s="8"/>
+      <c r="C201" s="8" t="s">
+        <v>487</v>
+      </c>
+      <c r="D201" s="8">
+        <v>1</v>
+      </c>
       <c r="E201" s="8"/>
       <c r="F201" s="8"/>
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A202" s="41"/>
-      <c r="B202" s="8"/>
-      <c r="C202" s="8"/>
-      <c r="D202" s="8"/>
+      <c r="B202" s="8" t="s">
+        <v>623</v>
+      </c>
+      <c r="C202" s="8" t="s">
+        <v>624</v>
+      </c>
+      <c r="D202" s="8">
+        <v>1</v>
+      </c>
       <c r="E202" s="8"/>
-      <c r="F202" s="8"/>
+      <c r="F202" s="8">
+        <v>360</v>
+      </c>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A203" s="41"/>
       <c r="B203" s="8"/>
-      <c r="C203" s="8"/>
-      <c r="D203" s="8"/>
+      <c r="C203" s="8" t="s">
+        <v>528</v>
+      </c>
+      <c r="D203" s="8">
+        <v>1</v>
+      </c>
       <c r="E203" s="8"/>
       <c r="F203" s="8"/>
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A204" s="41"/>
       <c r="B204" s="8"/>
-      <c r="C204" s="8"/>
-      <c r="D204" s="8"/>
+      <c r="C204" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="D204" s="8">
+        <v>1</v>
+      </c>
       <c r="E204" s="8"/>
       <c r="F204" s="8"/>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A205" s="41"/>
       <c r="B205" s="8"/>
-      <c r="C205" s="8"/>
-      <c r="D205" s="8"/>
+      <c r="C205" s="8" t="s">
+        <v>505</v>
+      </c>
+      <c r="D205" s="8">
+        <v>1</v>
+      </c>
       <c r="E205" s="8"/>
       <c r="F205" s="8"/>
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A206" s="41"/>
       <c r="B206" s="8"/>
-      <c r="C206" s="8"/>
-      <c r="D206" s="8"/>
+      <c r="C206" s="8" t="s">
+        <v>497</v>
+      </c>
+      <c r="D206" s="8">
+        <v>1</v>
+      </c>
       <c r="E206" s="8"/>
       <c r="F206" s="8"/>
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A207" s="41"/>
       <c r="B207" s="8"/>
-      <c r="C207" s="8"/>
-      <c r="D207" s="8"/>
+      <c r="C207" s="8" t="s">
+        <v>477</v>
+      </c>
+      <c r="D207" s="8">
+        <v>1</v>
+      </c>
       <c r="E207" s="8"/>
       <c r="F207" s="8"/>
     </row>
     <row r="208" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A208" s="41"/>
-      <c r="B208" s="8"/>
-      <c r="C208" s="8"/>
-      <c r="D208" s="8"/>
+      <c r="B208" s="8" t="s">
+        <v>624</v>
+      </c>
+      <c r="C208" s="8" t="s">
+        <v>625</v>
+      </c>
+      <c r="D208" s="8">
+        <v>1</v>
+      </c>
       <c r="E208" s="8"/>
-      <c r="F208" s="8"/>
+      <c r="F208" s="8">
+        <v>340</v>
+      </c>
     </row>
     <row r="209" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A209" s="41"/>
       <c r="B209" s="8"/>
-      <c r="C209" s="8"/>
-      <c r="D209" s="8"/>
+      <c r="C209" s="8" t="s">
+        <v>494</v>
+      </c>
+      <c r="D209" s="8">
+        <v>1</v>
+      </c>
       <c r="E209" s="8"/>
       <c r="F209" s="8"/>
     </row>
     <row r="210" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A210" s="41"/>
       <c r="B210" s="8"/>
-      <c r="C210" s="8"/>
-      <c r="D210" s="8"/>
+      <c r="C210" s="8" t="s">
+        <v>470</v>
+      </c>
+      <c r="D210" s="8">
+        <v>1</v>
+      </c>
       <c r="E210" s="8"/>
       <c r="F210" s="8"/>
     </row>
     <row r="211" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A211" s="41"/>
       <c r="B211" s="8"/>
-      <c r="C211" s="8"/>
-      <c r="D211" s="8"/>
+      <c r="C211" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="D211" s="8">
+        <v>1</v>
+      </c>
       <c r="E211" s="8"/>
       <c r="F211" s="8"/>
     </row>
     <row r="212" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A212" s="41"/>
       <c r="B212" s="8"/>
-      <c r="C212" s="8"/>
-      <c r="D212" s="8"/>
+      <c r="C212" s="8" t="s">
+        <v>436</v>
+      </c>
+      <c r="D212" s="8">
+        <v>1</v>
+      </c>
       <c r="E212" s="8"/>
       <c r="F212" s="8"/>
     </row>
     <row r="213" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A213" s="41"/>
       <c r="B213" s="8"/>
-      <c r="C213" s="8"/>
-      <c r="D213" s="8"/>
+      <c r="C213" s="8" t="s">
+        <v>536</v>
+      </c>
+      <c r="D213" s="8">
+        <v>1</v>
+      </c>
       <c r="E213" s="8"/>
       <c r="F213" s="8"/>
     </row>
     <row r="214" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A214" s="41"/>
-      <c r="B214" s="8"/>
-      <c r="C214" s="8"/>
-      <c r="D214" s="8"/>
+      <c r="B214" s="8" t="s">
+        <v>625</v>
+      </c>
+      <c r="C214" s="8" t="s">
+        <v>626</v>
+      </c>
+      <c r="D214" s="8">
+        <v>1</v>
+      </c>
       <c r="E214" s="8"/>
-      <c r="F214" s="8"/>
+      <c r="F214" s="8">
+        <v>320</v>
+      </c>
     </row>
     <row r="215" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A215" s="41"/>
       <c r="B215" s="8"/>
-      <c r="C215" s="8"/>
-      <c r="D215" s="8"/>
+      <c r="C215" s="8" t="s">
+        <v>466</v>
+      </c>
+      <c r="D215" s="8">
+        <v>1</v>
+      </c>
       <c r="E215" s="8"/>
       <c r="F215" s="8"/>
     </row>
     <row r="216" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A216" s="41"/>
       <c r="B216" s="8"/>
-      <c r="C216" s="8"/>
-      <c r="D216" s="8"/>
+      <c r="C216" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="D216" s="8">
+        <v>1</v>
+      </c>
       <c r="E216" s="8"/>
       <c r="F216" s="8"/>
     </row>
     <row r="217" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A217" s="41"/>
       <c r="B217" s="8"/>
-      <c r="C217" s="8"/>
-      <c r="D217" s="8"/>
+      <c r="C217" s="8" t="s">
+        <v>467</v>
+      </c>
+      <c r="D217" s="8">
+        <v>1</v>
+      </c>
       <c r="E217" s="8"/>
       <c r="F217" s="8"/>
     </row>
     <row r="218" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A218" s="41"/>
       <c r="B218" s="8"/>
-      <c r="C218" s="8"/>
-      <c r="D218" s="8"/>
+      <c r="C218" s="8" t="s">
+        <v>581</v>
+      </c>
+      <c r="D218" s="8">
+        <v>1</v>
+      </c>
       <c r="E218" s="8"/>
       <c r="F218" s="8"/>
     </row>
     <row r="219" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A219" s="41"/>
       <c r="B219" s="8"/>
-      <c r="C219" s="8"/>
-      <c r="D219" s="8"/>
+      <c r="C219" s="8" t="s">
+        <v>444</v>
+      </c>
+      <c r="D219" s="8">
+        <v>1</v>
+      </c>
       <c r="E219" s="8"/>
       <c r="F219" s="8"/>
     </row>

</xml_diff>